<commit_message>
chore(community): add contributor-management files
Adds the standard community-health files so outside contributors have a clear on-ramp:  - CONTRIBUTING.md  — dev setup, coding standards, commit conventions, PR checklist - CODE_OF_CONDUCT.md — Contributor Covenant 2.1 - SECURITY.md  — private vulnerability disclosure process - CHANGELOG.md — Keep-a-Changelog, seeded with 1.2.4 / 1.2.5 - .github/CODEOWNERS — default reviewers - .github/PULL_REQUEST_TEMPLATE.md — PR checklist - .github/ISSUE_TEMPLATE/{config.yml,bug_report.yml,feature_request.yml} - .github/workflows/ci.yml — lint + build on every PR, bundle artifact on push to main  README now links to CONTRIBUTING, SECURITY, CHANGELOG.
</commit_message>
<xml_diff>
--- a/test-harness/.tmp/aggregate-filled.xlsx
+++ b/test-harness/.tmp/aggregate-filled.xlsx
@@ -418,7 +418,7 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Generated: 2026-04-23T13:18:37.556Z</v>
+        <v>Generated: 2026-04-23T14:27:58.163Z</v>
       </c>
     </row>
     <row r="6">
@@ -772,18 +772,18 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Matoto MCHP</v>
+        <v>Masselleh MCHP</v>
       </c>
       <c r="B5" t="str">
-        <v>uGa5JtIMfRx</v>
+        <v>cag6vQQ9SQk</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Masselleh MCHP</v>
+        <v>Matoto MCHP</v>
       </c>
       <c r="B6" t="str">
-        <v>cag6vQQ9SQk</v>
+        <v>uGa5JtIMfRx</v>
       </c>
     </row>
     <row r="7">
@@ -1140,18 +1140,18 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Timbo CHP</v>
+        <v>SLRC (Mattru) Clinic</v>
       </c>
       <c r="B51" t="str">
-        <v>svCLFkT99Yx</v>
+        <v>T2Cn45nBY0u</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>SLRC (Mattru) Clinic</v>
+        <v>Timbo CHP</v>
       </c>
       <c r="B52" t="str">
-        <v>T2Cn45nBY0u</v>
+        <v>svCLFkT99Yx</v>
       </c>
     </row>
     <row r="53">
@@ -1180,18 +1180,18 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
-        <v>Banana Island MCHP</v>
+        <v>Rofutha MCHP</v>
       </c>
       <c r="B56" t="str">
-        <v>jjtzkzrmG7s</v>
+        <v>G5FuODAbH6X</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="str">
-        <v>Rofutha MCHP</v>
+        <v>Banana Island MCHP</v>
       </c>
       <c r="B57" t="str">
-        <v>G5FuODAbH6X</v>
+        <v>jjtzkzrmG7s</v>
       </c>
     </row>
     <row r="58">
@@ -1372,18 +1372,18 @@
     </row>
     <row r="80">
       <c r="A80" t="str">
-        <v>Nekabo CHC</v>
+        <v>Kissy Town CHP</v>
       </c>
       <c r="B80" t="str">
-        <v>L4Tw4NlaMjn</v>
+        <v>lmNWdmeOYmV</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="str">
-        <v>Kissy Town CHP</v>
+        <v>Nekabo CHC</v>
       </c>
       <c r="B81" t="str">
-        <v>lmNWdmeOYmV</v>
+        <v>L4Tw4NlaMjn</v>
       </c>
     </row>
     <row r="82">
@@ -1612,18 +1612,18 @@
     </row>
     <row r="110">
       <c r="A110" t="str">
-        <v>Stella Maries Clinic</v>
+        <v>Yemoh Town CHC</v>
       </c>
       <c r="B110" t="str">
-        <v>Ea3j0kUvyWg</v>
+        <v>RhJbg8UD75Q</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="str">
-        <v>Yemoh Town CHC</v>
+        <v>Stella Maries Clinic</v>
       </c>
       <c r="B111" t="str">
-        <v>RhJbg8UD75Q</v>
+        <v>Ea3j0kUvyWg</v>
       </c>
     </row>
     <row r="112">
@@ -1676,18 +1676,18 @@
     </row>
     <row r="118">
       <c r="A118" t="str">
-        <v>Minah MCHP</v>
+        <v>Mogbasske CHP</v>
       </c>
       <c r="B118" t="str">
-        <v>ZW3XCXXiLcO</v>
+        <v>DZaJmtlaBMl</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="str">
-        <v>Mogbasske CHP</v>
+        <v>Minah MCHP</v>
       </c>
       <c r="B119" t="str">
-        <v>DZaJmtlaBMl</v>
+        <v>ZW3XCXXiLcO</v>
       </c>
     </row>
     <row r="120">
@@ -1796,26 +1796,26 @@
     </row>
     <row r="133">
       <c r="A133" t="str">
-        <v>Kaponkie MCHP</v>
+        <v>Woyama MCHP</v>
       </c>
       <c r="B133" t="str">
-        <v>Crgx572DnXR</v>
+        <v>fPe1l06MurL</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="str">
-        <v>Woyama MCHP</v>
+        <v>Mabora MCHP</v>
       </c>
       <c r="B134" t="str">
-        <v>fPe1l06MurL</v>
+        <v>fmkqsEx6MRo</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="str">
-        <v>Mabora MCHP</v>
+        <v>Kaponkie MCHP</v>
       </c>
       <c r="B135" t="str">
-        <v>fmkqsEx6MRo</v>
+        <v>Crgx572DnXR</v>
       </c>
     </row>
     <row r="136">
@@ -1852,18 +1852,18 @@
     </row>
     <row r="140">
       <c r="A140" t="str">
-        <v>Masankoro MCHP</v>
+        <v>Small Sefadu MCHP</v>
       </c>
       <c r="B140" t="str">
-        <v>l3jnkNNpoD8</v>
+        <v>ncGs9vXS36w</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="str">
-        <v>Small Sefadu MCHP</v>
+        <v>Masankoro MCHP</v>
       </c>
       <c r="B141" t="str">
-        <v>ncGs9vXS36w</v>
+        <v>l3jnkNNpoD8</v>
       </c>
     </row>
     <row r="142">
@@ -1924,18 +1924,18 @@
     </row>
     <row r="149">
       <c r="A149" t="str">
-        <v>Scan Drive MCHP</v>
+        <v>Kokoru CHP</v>
       </c>
       <c r="B149" t="str">
-        <v>u1eQDDtKqm7</v>
+        <v>F2TAF765q1b</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="str">
-        <v>Kokoru CHP</v>
+        <v>Scan Drive MCHP</v>
       </c>
       <c r="B150" t="str">
-        <v>F2TAF765q1b</v>
+        <v>u1eQDDtKqm7</v>
       </c>
     </row>
     <row r="151">
@@ -1980,18 +1980,18 @@
     </row>
     <row r="156">
       <c r="A156" t="str">
-        <v>Bambawolo CHP</v>
+        <v>Madina (Malema) MCHP</v>
       </c>
       <c r="B156" t="str">
-        <v>TNbHYOuQi8s</v>
+        <v>SFQigiC2ISS</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="str">
-        <v>Madina (Malema) MCHP</v>
+        <v>Bambawolo CHP</v>
       </c>
       <c r="B157" t="str">
-        <v>SFQigiC2ISS</v>
+        <v>TNbHYOuQi8s</v>
       </c>
     </row>
     <row r="158">
@@ -2140,18 +2140,18 @@
     </row>
     <row r="176">
       <c r="A176" t="str">
-        <v>Masongbo CHC</v>
+        <v>Mabineh MCHP</v>
       </c>
       <c r="B176" t="str">
-        <v>uRQj8WRK0Py</v>
+        <v>mc3jvzpzSi4</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="str">
-        <v>Mabineh MCHP</v>
+        <v>Masongbo CHC</v>
       </c>
       <c r="B177" t="str">
-        <v>mc3jvzpzSi4</v>
+        <v>uRQj8WRK0Py</v>
       </c>
     </row>
     <row r="178">
@@ -2356,18 +2356,18 @@
     </row>
     <row r="203">
       <c r="A203" t="str">
-        <v>Masumbrie MCHP</v>
+        <v>Worreh MCHP</v>
       </c>
       <c r="B203" t="str">
-        <v>flJbtXOQ4ha</v>
+        <v>VSwnkMSAdp7</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="str">
-        <v>Worreh MCHP</v>
+        <v>Masumbrie MCHP</v>
       </c>
       <c r="B204" t="str">
-        <v>VSwnkMSAdp7</v>
+        <v>flJbtXOQ4ha</v>
       </c>
     </row>
     <row r="205">
@@ -2444,18 +2444,18 @@
     </row>
     <row r="214">
       <c r="A214" t="str">
-        <v>Mamanso Kafla MCHP</v>
+        <v>Kindoyal Hospital</v>
       </c>
       <c r="B214" t="str">
-        <v>T1lTKu6zkHN</v>
+        <v>uROAmk9ymNE</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="str">
-        <v>Kindoyal Hospital</v>
+        <v>Mamanso Kafla MCHP</v>
       </c>
       <c r="B215" t="str">
-        <v>uROAmk9ymNE</v>
+        <v>T1lTKu6zkHN</v>
       </c>
     </row>
     <row r="216">
@@ -2524,26 +2524,26 @@
     </row>
     <row r="224">
       <c r="A224" t="str">
-        <v>Kanekor MCHP</v>
+        <v>Magbassabana MCHP</v>
       </c>
       <c r="B224" t="str">
-        <v>tXL6C7P0ObJ</v>
+        <v>bf6PXrSNMKK</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="str">
-        <v>Bumpeh River CHP</v>
+        <v>Kanekor MCHP</v>
       </c>
       <c r="B225" t="str">
-        <v>mkIugjeYSjE</v>
+        <v>tXL6C7P0ObJ</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="str">
-        <v>Magbassabana MCHP</v>
+        <v>Bumpeh River CHP</v>
       </c>
       <c r="B226" t="str">
-        <v>bf6PXrSNMKK</v>
+        <v>mkIugjeYSjE</v>
       </c>
     </row>
     <row r="227">
@@ -2612,18 +2612,18 @@
     </row>
     <row r="235">
       <c r="A235" t="str">
-        <v>Delken MCHP</v>
+        <v>Jangalor MCHP</v>
       </c>
       <c r="B235" t="str">
-        <v>sSgOnY1Xqd9</v>
+        <v>qzm5ww3U0vz</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="str">
-        <v>Jangalor MCHP</v>
+        <v>Delken MCHP</v>
       </c>
       <c r="B236" t="str">
-        <v>qzm5ww3U0vz</v>
+        <v>sSgOnY1Xqd9</v>
       </c>
     </row>
     <row r="237">
@@ -2956,18 +2956,18 @@
     </row>
     <row r="278">
       <c r="A278" t="str">
-        <v>Numea CHC</v>
+        <v>Tongoro MCHP</v>
       </c>
       <c r="B278" t="str">
-        <v>PduUQmdt0pB</v>
+        <v>iIpPPnnzDo6</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="str">
-        <v>Tongoro MCHP</v>
+        <v>Numea CHC</v>
       </c>
       <c r="B279" t="str">
-        <v>iIpPPnnzDo6</v>
+        <v>PduUQmdt0pB</v>
       </c>
     </row>
     <row r="280">
@@ -3052,34 +3052,34 @@
     </row>
     <row r="290">
       <c r="A290" t="str">
-        <v>Senjekoro MCHP</v>
+        <v>Bo Govt. Hosp.</v>
       </c>
       <c r="B290" t="str">
-        <v>tcEjL7gmFJL</v>
+        <v>rZxk3S0qN63</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="str">
-        <v>Bo Govt. Hosp.</v>
+        <v>Senjekoro MCHP</v>
       </c>
       <c r="B291" t="str">
-        <v>rZxk3S0qN63</v>
+        <v>tcEjL7gmFJL</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="str">
-        <v>UFC Bonthe</v>
+        <v>Tonkomba MCHP</v>
       </c>
       <c r="B292" t="str">
-        <v>gGv9ATEs68L</v>
+        <v>xIMxph4NMP1</v>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="str">
-        <v>Tonkomba MCHP</v>
+        <v>UFC Bonthe</v>
       </c>
       <c r="B293" t="str">
-        <v>xIMxph4NMP1</v>
+        <v>gGv9ATEs68L</v>
       </c>
     </row>
     <row r="294">
@@ -3172,18 +3172,18 @@
     </row>
     <row r="305">
       <c r="A305" t="str">
-        <v>Mercy Ship ACFC</v>
+        <v>Fatibra CHP</v>
       </c>
       <c r="B305" t="str">
-        <v>xO9WbCvFq5k</v>
+        <v>jfV49JGnYKF</v>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="str">
-        <v>Fatibra CHP</v>
+        <v>Mercy Ship ACFC</v>
       </c>
       <c r="B306" t="str">
-        <v>jfV49JGnYKF</v>
+        <v>xO9WbCvFq5k</v>
       </c>
     </row>
     <row r="307">
@@ -3420,18 +3420,18 @@
     </row>
     <row r="336">
       <c r="A336" t="str">
-        <v>Makobeh MCHP</v>
+        <v>Yataya CHP</v>
       </c>
       <c r="B336" t="str">
-        <v>iMDr2FG7i8Q</v>
+        <v>MErVkzdbsP5</v>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="str">
-        <v>Yataya CHP</v>
+        <v>Makobeh MCHP</v>
       </c>
       <c r="B337" t="str">
-        <v>MErVkzdbsP5</v>
+        <v>iMDr2FG7i8Q</v>
       </c>
     </row>
     <row r="338">
@@ -3444,18 +3444,18 @@
     </row>
     <row r="339">
       <c r="A339" t="str">
-        <v>Mabayo MCHP</v>
+        <v>Dankawalie MCHP</v>
       </c>
       <c r="B339" t="str">
-        <v>Xzxy8NuVsLp</v>
+        <v>DErmFP7bri7</v>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="str">
-        <v>Dankawalie MCHP</v>
+        <v>Mabayo MCHP</v>
       </c>
       <c r="B340" t="str">
-        <v>DErmFP7bri7</v>
+        <v>Xzxy8NuVsLp</v>
       </c>
     </row>
     <row r="341">
@@ -3516,18 +3516,18 @@
     </row>
     <row r="348">
       <c r="A348" t="str">
-        <v>Masamboi MCHP</v>
+        <v>Gbetema MCHP (Fiama)</v>
       </c>
       <c r="B348" t="str">
-        <v>Hu31NCRjZlj</v>
+        <v>as1dnmlXLzG</v>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="str">
-        <v>Gbetema MCHP (Fiama)</v>
+        <v>Masamboi MCHP</v>
       </c>
       <c r="B349" t="str">
-        <v>as1dnmlXLzG</v>
+        <v>Hu31NCRjZlj</v>
       </c>
     </row>
     <row r="350">
@@ -4356,18 +4356,18 @@
     </row>
     <row r="453">
       <c r="A453" t="str">
-        <v>Kpetema MCHP</v>
+        <v>Ngueh MCHP</v>
       </c>
       <c r="B453" t="str">
-        <v>kDxbU1uSBFh</v>
+        <v>Vw4Uv6UPIPC</v>
       </c>
     </row>
     <row r="454">
       <c r="A454" t="str">
-        <v>Ngueh MCHP</v>
+        <v>Kpetema MCHP</v>
       </c>
       <c r="B454" t="str">
-        <v>Vw4Uv6UPIPC</v>
+        <v>kDxbU1uSBFh</v>
       </c>
     </row>
     <row r="455">
@@ -4516,18 +4516,18 @@
     </row>
     <row r="473">
       <c r="A473" t="str">
-        <v>Praise Foundation CHC</v>
+        <v>Mayassoh MCHP</v>
       </c>
       <c r="B473" t="str">
-        <v>wtdBuXDwZYQ</v>
+        <v>Z8Cm76B2726</v>
       </c>
     </row>
     <row r="474">
       <c r="A474" t="str">
-        <v>Mayassoh MCHP</v>
+        <v>Praise Foundation CHC</v>
       </c>
       <c r="B474" t="str">
-        <v>Z8Cm76B2726</v>
+        <v>wtdBuXDwZYQ</v>
       </c>
     </row>
     <row r="475">
@@ -4804,18 +4804,18 @@
     </row>
     <row r="509">
       <c r="A509" t="str">
-        <v>Rosint Buya MCHP</v>
+        <v>Sahn Bumpe MCHP</v>
       </c>
       <c r="B509" t="str">
-        <v>el8sgzyHuEe</v>
+        <v>NDqR2cWlVy3</v>
       </c>
     </row>
     <row r="510">
       <c r="A510" t="str">
-        <v>Sahn Bumpe MCHP</v>
+        <v>Rosint Buya MCHP</v>
       </c>
       <c r="B510" t="str">
-        <v>NDqR2cWlVy3</v>
+        <v>el8sgzyHuEe</v>
       </c>
     </row>
     <row r="511">
@@ -5004,18 +5004,18 @@
     </row>
     <row r="534">
       <c r="A534" t="str">
-        <v>Gbangba MCHP</v>
+        <v>Wai MCHP</v>
       </c>
       <c r="B534" t="str">
-        <v>r93q83kZoR9</v>
+        <v>zCSWBz2pyMd</v>
       </c>
     </row>
     <row r="535">
       <c r="A535" t="str">
-        <v>Wai MCHP</v>
+        <v>Gbangba MCHP</v>
       </c>
       <c r="B535" t="str">
-        <v>zCSWBz2pyMd</v>
+        <v>r93q83kZoR9</v>
       </c>
     </row>
     <row r="536">
@@ -5404,18 +5404,18 @@
     </row>
     <row r="584">
       <c r="A584" t="str">
-        <v>kamba mamudia</v>
+        <v>Madina (BUM) CHC</v>
       </c>
       <c r="B584" t="str">
-        <v>zO5hgxxfU4T</v>
+        <v>gE3gEGZbQMi</v>
       </c>
     </row>
     <row r="585">
       <c r="A585" t="str">
-        <v>Madina (BUM) CHC</v>
+        <v>kamba mamudia</v>
       </c>
       <c r="B585" t="str">
-        <v>gE3gEGZbQMi</v>
+        <v>zO5hgxxfU4T</v>
       </c>
     </row>
     <row r="586">
@@ -5564,18 +5564,18 @@
     </row>
     <row r="604">
       <c r="A604" t="str">
-        <v>Gbendembu Wesleyan CHC</v>
+        <v>Bandasuma Fiama MCHP</v>
       </c>
       <c r="B604" t="str">
-        <v>YAuJ3fyoEuI</v>
+        <v>aF6iPGbrcRk</v>
       </c>
     </row>
     <row r="605">
       <c r="A605" t="str">
-        <v>Bandasuma Fiama MCHP</v>
+        <v>Gbendembu Wesleyan CHC</v>
       </c>
       <c r="B605" t="str">
-        <v>aF6iPGbrcRk</v>
+        <v>YAuJ3fyoEuI</v>
       </c>
     </row>
     <row r="606">
@@ -5764,18 +5764,18 @@
     </row>
     <row r="629">
       <c r="A629" t="str">
-        <v>Wordu CHP</v>
+        <v>Robat MCHP</v>
       </c>
       <c r="B629" t="str">
-        <v>bW5BaqrBM4K</v>
+        <v>gP6hn503KUX</v>
       </c>
     </row>
     <row r="630">
       <c r="A630" t="str">
-        <v>Robat MCHP</v>
+        <v>Wordu CHP</v>
       </c>
       <c r="B630" t="str">
-        <v>gP6hn503KUX</v>
+        <v>bW5BaqrBM4K</v>
       </c>
     </row>
     <row r="631">
@@ -5796,18 +5796,18 @@
     </row>
     <row r="633">
       <c r="A633" t="str">
-        <v>SLRCS (Nongowa) clinic</v>
+        <v>Wellbody MCHP</v>
       </c>
       <c r="B633" t="str">
-        <v>Vnc2qIRLbyw</v>
+        <v>XuGfiry96Bg</v>
       </c>
     </row>
     <row r="634">
       <c r="A634" t="str">
-        <v>Wellbody MCHP</v>
+        <v>SLRCS (Nongowa) clinic</v>
       </c>
       <c r="B634" t="str">
-        <v>XuGfiry96Bg</v>
+        <v>Vnc2qIRLbyw</v>
       </c>
     </row>
     <row r="635">
@@ -5860,18 +5860,18 @@
     </row>
     <row r="641">
       <c r="A641" t="str">
-        <v>Bendu Mameima CHC</v>
+        <v>Kamba MCHP</v>
       </c>
       <c r="B641" t="str">
-        <v>amgb83zVxp5</v>
+        <v>cJ7omISg7gG</v>
       </c>
     </row>
     <row r="642">
       <c r="A642" t="str">
-        <v>Kamba MCHP</v>
+        <v>Bendu Mameima CHC</v>
       </c>
       <c r="B642" t="str">
-        <v>cJ7omISg7gG</v>
+        <v>amgb83zVxp5</v>
       </c>
     </row>
     <row r="643">
@@ -6572,18 +6572,18 @@
     </row>
     <row r="730">
       <c r="A730" t="str">
-        <v>Kania (Masungbala) MCHP</v>
+        <v>Musaia CHP</v>
       </c>
       <c r="B730" t="str">
-        <v>RNGpZqutw3Y</v>
+        <v>sTOXJA2KcY2</v>
       </c>
     </row>
     <row r="731">
       <c r="A731" t="str">
-        <v>Musaia CHP</v>
+        <v>Kania (Masungbala) MCHP</v>
       </c>
       <c r="B731" t="str">
-        <v>sTOXJA2KcY2</v>
+        <v>RNGpZqutw3Y</v>
       </c>
     </row>
     <row r="732">
@@ -6684,18 +6684,18 @@
     </row>
     <row r="744">
       <c r="A744" t="str">
-        <v>Koakor MCHP</v>
+        <v>Sumbuya CHC</v>
       </c>
       <c r="B744" t="str">
-        <v>EQc3n1juPFn</v>
+        <v>W2KnxOMvmgE</v>
       </c>
     </row>
     <row r="745">
       <c r="A745" t="str">
-        <v>Sumbuya CHC</v>
+        <v>Koakor MCHP</v>
       </c>
       <c r="B745" t="str">
-        <v>W2KnxOMvmgE</v>
+        <v>EQc3n1juPFn</v>
       </c>
     </row>
     <row r="746">
@@ -6916,18 +6916,18 @@
     </row>
     <row r="773">
       <c r="A773" t="str">
-        <v>Gissiwolo MCHP</v>
+        <v>Rothatha MCHP</v>
       </c>
       <c r="B773" t="str">
-        <v>AekX8HBymng</v>
+        <v>KaevAHPgkA8</v>
       </c>
     </row>
     <row r="774">
       <c r="A774" t="str">
-        <v>Rothatha MCHP</v>
+        <v>Gissiwolo MCHP</v>
       </c>
       <c r="B774" t="str">
-        <v>KaevAHPgkA8</v>
+        <v>AekX8HBymng</v>
       </c>
     </row>
     <row r="775">
@@ -6940,50 +6940,50 @@
     </row>
     <row r="776">
       <c r="A776" t="str">
-        <v>Sebengu MCHP</v>
+        <v>Sengama MCHP</v>
       </c>
       <c r="B776" t="str">
-        <v>Jd7G0NYBTx1</v>
+        <v>MBtmOhLs7y1</v>
       </c>
     </row>
     <row r="777">
       <c r="A777" t="str">
-        <v>Sengama MCHP</v>
+        <v>Sebengu MCHP</v>
       </c>
       <c r="B777" t="str">
-        <v>MBtmOhLs7y1</v>
+        <v>Jd7G0NYBTx1</v>
       </c>
     </row>
     <row r="778">
       <c r="A778" t="str">
-        <v>Kpayama 1 MCHP</v>
+        <v>Ngiehun (Lower Bambara) MCHP</v>
       </c>
       <c r="B778" t="str">
-        <v>So2b8zJfcMa</v>
+        <v>m21WB5iqHAb</v>
       </c>
     </row>
     <row r="779">
       <c r="A779" t="str">
-        <v>Ngiehun (Lower Bambara) MCHP</v>
+        <v>Kpayama 1 MCHP</v>
       </c>
       <c r="B779" t="str">
-        <v>m21WB5iqHAb</v>
+        <v>So2b8zJfcMa</v>
       </c>
     </row>
     <row r="780">
       <c r="A780" t="str">
-        <v>Gbandiwulo CHP</v>
+        <v>Manewa MCHP</v>
       </c>
       <c r="B780" t="str">
-        <v>Vw6CNyFUeh9</v>
+        <v>CTnuuI55SOj</v>
       </c>
     </row>
     <row r="781">
       <c r="A781" t="str">
-        <v>Manewa MCHP</v>
+        <v>Gbandiwulo CHP</v>
       </c>
       <c r="B781" t="str">
-        <v>CTnuuI55SOj</v>
+        <v>Vw6CNyFUeh9</v>
       </c>
     </row>
     <row r="782">
@@ -6996,18 +6996,18 @@
     </row>
     <row r="783">
       <c r="A783" t="str">
-        <v>Gbindi CHP</v>
+        <v>Sandaru (Gaura) MCHP</v>
       </c>
       <c r="B783" t="str">
-        <v>LFpl1falVZi</v>
+        <v>hTGeTrwzrPi</v>
       </c>
     </row>
     <row r="784">
       <c r="A784" t="str">
-        <v>Sandaru (Gaura) MCHP</v>
+        <v>Gbindi CHP</v>
       </c>
       <c r="B784" t="str">
-        <v>hTGeTrwzrPi</v>
+        <v>LFpl1falVZi</v>
       </c>
     </row>
     <row r="785">
@@ -7044,18 +7044,18 @@
     </row>
     <row r="789">
       <c r="A789" t="str">
-        <v>Mandema CHP</v>
+        <v>Torkpumbu MCHP</v>
       </c>
       <c r="B789" t="str">
-        <v>WerHl8SDtRU</v>
+        <v>RJpiHpefEUw</v>
       </c>
     </row>
     <row r="790">
       <c r="A790" t="str">
-        <v>Torkpumbu MCHP</v>
+        <v>Mandema CHP</v>
       </c>
       <c r="B790" t="str">
-        <v>RJpiHpefEUw</v>
+        <v>WerHl8SDtRU</v>
       </c>
     </row>
     <row r="791">
@@ -7516,26 +7516,26 @@
     </row>
     <row r="848">
       <c r="A848" t="str">
-        <v>Needy CHC</v>
+        <v>Sienga CHP</v>
       </c>
       <c r="B848" t="str">
-        <v>UOJlcpPnBat</v>
+        <v>a1E6QWBTEwX</v>
       </c>
     </row>
     <row r="849">
       <c r="A849" t="str">
-        <v>Sienga CHP</v>
+        <v>Needy CHC</v>
       </c>
       <c r="B849" t="str">
-        <v>a1E6QWBTEwX</v>
+        <v>UOJlcpPnBat</v>
       </c>
     </row>
     <row r="850">
       <c r="A850" t="str">
-        <v>Mayakie MCHP</v>
+        <v>New Maforkie CHP</v>
       </c>
       <c r="B850" t="str">
-        <v>R0CmUlFULXg</v>
+        <v>lzz1UhTzO4E</v>
       </c>
     </row>
     <row r="851">
@@ -7548,10 +7548,10 @@
     </row>
     <row r="852">
       <c r="A852" t="str">
-        <v>New Maforkie CHP</v>
+        <v>Mayakie MCHP</v>
       </c>
       <c r="B852" t="str">
-        <v>lzz1UhTzO4E</v>
+        <v>R0CmUlFULXg</v>
       </c>
     </row>
     <row r="853">
@@ -7684,18 +7684,18 @@
     </row>
     <row r="869">
       <c r="A869" t="str">
-        <v>Njama MCHP</v>
+        <v>Bongor MCHP</v>
       </c>
       <c r="B869" t="str">
-        <v>WMj6mBDw76A</v>
+        <v>zAyK28LLaez</v>
       </c>
     </row>
     <row r="870">
       <c r="A870" t="str">
-        <v>Bongor MCHP</v>
+        <v>Njama MCHP</v>
       </c>
       <c r="B870" t="str">
-        <v>zAyK28LLaez</v>
+        <v>WMj6mBDw76A</v>
       </c>
     </row>
     <row r="871">
@@ -7708,18 +7708,18 @@
     </row>
     <row r="872">
       <c r="A872" t="str">
-        <v>Konjo MCHP</v>
+        <v>SLRCS (Freetown) Clinic</v>
       </c>
       <c r="B872" t="str">
-        <v>d7hw1ababST</v>
+        <v>EmTN0L4EAVi</v>
       </c>
     </row>
     <row r="873">
       <c r="A873" t="str">
-        <v>SLRCS (Freetown) Clinic</v>
+        <v>Konjo MCHP</v>
       </c>
       <c r="B873" t="str">
-        <v>EmTN0L4EAVi</v>
+        <v>d7hw1ababST</v>
       </c>
     </row>
     <row r="874">
@@ -7804,18 +7804,18 @@
     </row>
     <row r="884">
       <c r="A884" t="str">
-        <v>Kambama CHP</v>
+        <v>Sandayeima MCHP</v>
       </c>
       <c r="B884" t="str">
-        <v>mYMJHVqdBKt</v>
+        <v>oUR5HPmim7E</v>
       </c>
     </row>
     <row r="885">
       <c r="A885" t="str">
-        <v>Sandayeima MCHP</v>
+        <v>Kambama CHP</v>
       </c>
       <c r="B885" t="str">
-        <v>oUR5HPmim7E</v>
+        <v>mYMJHVqdBKt</v>
       </c>
     </row>
     <row r="886">
@@ -8212,18 +8212,18 @@
     </row>
     <row r="935">
       <c r="A935" t="str">
-        <v>Mende Buima MCHP</v>
+        <v>Tissana MCHP</v>
       </c>
       <c r="B935" t="str">
-        <v>NnGUNkc5Zq8</v>
+        <v>SptGAcmbgPz</v>
       </c>
     </row>
     <row r="936">
       <c r="A936" t="str">
-        <v>Tissana MCHP</v>
+        <v>Mende Buima MCHP</v>
       </c>
       <c r="B936" t="str">
-        <v>SptGAcmbgPz</v>
+        <v>NnGUNkc5Zq8</v>
       </c>
     </row>
     <row r="937">
@@ -8516,18 +8516,18 @@
     </row>
     <row r="973">
       <c r="A973" t="str">
-        <v>Kondeya (Sandor) MCHP</v>
+        <v>Mokorbu MCHP</v>
       </c>
       <c r="B973" t="str">
-        <v>e5sGsWLEn3k</v>
+        <v>cHqboEGRUiY</v>
       </c>
     </row>
     <row r="974">
       <c r="A974" t="str">
-        <v>Mokorbu MCHP</v>
+        <v>Kondeya (Sandor) MCHP</v>
       </c>
       <c r="B974" t="str">
-        <v>cHqboEGRUiY</v>
+        <v>e5sGsWLEn3k</v>
       </c>
     </row>
     <row r="975">
@@ -8612,26 +8612,26 @@
     </row>
     <row r="985">
       <c r="A985" t="str">
-        <v>Mabang MCHP</v>
+        <v>Mano Yorgbo MCHP</v>
       </c>
       <c r="B985" t="str">
-        <v>fCFdj2T0Bq1</v>
+        <v>KvE0PYQzXMM</v>
       </c>
     </row>
     <row r="986">
       <c r="A986" t="str">
-        <v>Mano Yorgbo MCHP</v>
+        <v>Gloucester CHP</v>
       </c>
       <c r="B986" t="str">
-        <v>KvE0PYQzXMM</v>
+        <v>HTDuY3uxj6u</v>
       </c>
     </row>
     <row r="987">
       <c r="A987" t="str">
-        <v>Gloucester CHP</v>
+        <v>Mabang MCHP</v>
       </c>
       <c r="B987" t="str">
-        <v>HTDuY3uxj6u</v>
+        <v>fCFdj2T0Bq1</v>
       </c>
     </row>
     <row r="988">
@@ -8924,18 +8924,18 @@
     </row>
     <row r="1024">
       <c r="A1024" t="str">
-        <v>Laleihun Kovoma CHC</v>
+        <v>Sumbaria MCHP</v>
       </c>
       <c r="B1024" t="str">
-        <v>N3tpEjZcPm9</v>
+        <v>GvstqlRRnpV</v>
       </c>
     </row>
     <row r="1025">
       <c r="A1025" t="str">
-        <v>Sumbaria MCHP</v>
+        <v>Laleihun Kovoma CHC</v>
       </c>
       <c r="B1025" t="str">
-        <v>GvstqlRRnpV</v>
+        <v>N3tpEjZcPm9</v>
       </c>
     </row>
     <row r="1026">
@@ -9060,10 +9060,10 @@
     </row>
     <row r="1041">
       <c r="A1041" t="str">
-        <v>Mosanda CHP</v>
+        <v>Pewama CHP</v>
       </c>
       <c r="B1041" t="str">
-        <v>cDRQOxX1wHO</v>
+        <v>nbMpoRiVRWd</v>
       </c>
     </row>
     <row r="1042">
@@ -9076,10 +9076,10 @@
     </row>
     <row r="1043">
       <c r="A1043" t="str">
-        <v>Pewama CHP</v>
+        <v>Mosanda CHP</v>
       </c>
       <c r="B1043" t="str">
-        <v>nbMpoRiVRWd</v>
+        <v>cDRQOxX1wHO</v>
       </c>
     </row>
     <row r="1044">
@@ -9140,18 +9140,18 @@
     </row>
     <row r="1051">
       <c r="A1051" t="str">
-        <v>Komendeh (Nongowa) MCHP</v>
+        <v>Rolembray MCHP</v>
       </c>
       <c r="B1051" t="str">
-        <v>NqwvaQC1ni4</v>
+        <v>nZblzPvJ5UW</v>
       </c>
     </row>
     <row r="1052">
       <c r="A1052" t="str">
-        <v>Rolembray MCHP</v>
+        <v>Komendeh (Nongowa) MCHP</v>
       </c>
       <c r="B1052" t="str">
-        <v>nZblzPvJ5UW</v>
+        <v>NqwvaQC1ni4</v>
       </c>
     </row>
     <row r="1053">
@@ -9228,18 +9228,18 @@
     </row>
     <row r="1062">
       <c r="A1062" t="str">
-        <v>Yele CHC</v>
+        <v>Mabolleh MCHP</v>
       </c>
       <c r="B1062" t="str">
-        <v>sesv0eXljBq</v>
+        <v>PybxeRWVSrI</v>
       </c>
     </row>
     <row r="1063">
       <c r="A1063" t="str">
-        <v>Mabolleh MCHP</v>
+        <v>Yele CHC</v>
       </c>
       <c r="B1063" t="str">
-        <v>PybxeRWVSrI</v>
+        <v>sesv0eXljBq</v>
       </c>
     </row>
     <row r="1064">
@@ -9516,18 +9516,18 @@
     </row>
     <row r="1098">
       <c r="A1098" t="str">
-        <v>Gbalan Thallan MCHP</v>
+        <v>Tonko Maternity Clinic</v>
       </c>
       <c r="B1098" t="str">
-        <v>FsunWIQLXoF</v>
+        <v>uNEhNuBUr0i</v>
       </c>
     </row>
     <row r="1099">
       <c r="A1099" t="str">
-        <v>Tonko Maternity Clinic</v>
+        <v>Gbalan Thallan MCHP</v>
       </c>
       <c r="B1099" t="str">
-        <v>uNEhNuBUr0i</v>
+        <v>FsunWIQLXoF</v>
       </c>
     </row>
     <row r="1100">
@@ -9644,18 +9644,18 @@
     </row>
     <row r="1114">
       <c r="A1114" t="str">
-        <v>Bumban MCHP</v>
+        <v>Tagrin CHC</v>
       </c>
       <c r="B1114" t="str">
-        <v>OI0BQUurVFS</v>
+        <v>O63vIA5MVn6</v>
       </c>
     </row>
     <row r="1115">
       <c r="A1115" t="str">
-        <v>Tagrin CHC</v>
+        <v>Bumban MCHP</v>
       </c>
       <c r="B1115" t="str">
-        <v>O63vIA5MVn6</v>
+        <v>OI0BQUurVFS</v>
       </c>
     </row>
     <row r="1116">
@@ -9804,18 +9804,18 @@
     </row>
     <row r="1134">
       <c r="A1134" t="str">
-        <v>Gbongeima MCHP</v>
+        <v>Lion for Lion Clinic</v>
       </c>
       <c r="B1134" t="str">
-        <v>rebbn0ooFSO</v>
+        <v>cZxP4NE5O9z</v>
       </c>
     </row>
     <row r="1135">
       <c r="A1135" t="str">
-        <v>Lion for Lion Clinic</v>
+        <v>Gbongeima MCHP</v>
       </c>
       <c r="B1135" t="str">
-        <v>cZxP4NE5O9z</v>
+        <v>rebbn0ooFSO</v>
       </c>
     </row>
     <row r="1136">
@@ -10052,18 +10052,18 @@
     </row>
     <row r="1165">
       <c r="A1165" t="str">
-        <v>Mabang CHC</v>
+        <v>Gbonkobana CHP</v>
       </c>
       <c r="B1165" t="str">
-        <v>Ahh47q8AkId</v>
+        <v>BXJnMD2eJAx</v>
       </c>
     </row>
     <row r="1166">
       <c r="A1166" t="str">
-        <v>Gbonkobana CHP</v>
+        <v>Mabang CHC</v>
       </c>
       <c r="B1166" t="str">
-        <v>BXJnMD2eJAx</v>
+        <v>Ahh47q8AkId</v>
       </c>
     </row>
     <row r="1167">

</xml_diff>